<commit_message>
Quotation: set units per box from founder (180ML 50, 750ML 16, 500ML 16)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WKbZ2PH3fH4AvF1j5yCwZ2
</commit_message>
<xml_diff>
--- a/deliverables/songyoungshin/현대그린푸드_견적서_송영신목장.xlsx
+++ b/deliverables/songyoungshin/현대그린푸드_견적서_송영신목장.xlsx
@@ -1334,7 +1334,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="G7" s="22" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="S7" s="43" t="inlineStr">
         <is>
-          <t>※ 직매입 · 냉장 4℃ · 저온살균 A2 저지 우유 · 원가는 M/G 30% 기준 제안(안) · 박스입수·유통기한 확인 필요</t>
+          <t>※ 직매입 · 냉장 4℃ · 저온살균 A2 저지 우유 · 원가는 M/G 30% 기준 제안(안) · 유통기한 확인 필요</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G8" s="22" t="inlineStr">
         <is>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="S8" s="43" t="inlineStr">
         <is>
-          <t>※ 직매입 · 냉장 4℃ · 매가·원가 제안(안, 180ML 대비 mL당 약 25% 인하) · 박스입수·유통기한 확인 필요</t>
+          <t>※ 직매입 · 냉장 4℃ · 매가·원가 제안(안, 180ML 대비 mL당 약 25% 인하) · 유통기한 확인 필요</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="G9" s="22" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="S9" s="43" t="inlineStr">
         <is>
-          <t>※ 직매입 · 냉장 4℃ · 무가당 플레인(과세) · 매가·원가 제안(안) · 박스입수·유통기한 확인 필요</t>
+          <t>※ 직매입 · 냉장 4℃ · 무가당 플레인(과세) · 매가·원가 제안(안) · 유통기한 확인 필요</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G10" s="22" t="inlineStr">
         <is>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="S10" s="43" t="inlineStr">
         <is>
-          <t>※ 직매입 · 냉장 4℃ · 무가당 플레인(과세) · 매가·원가 제안(안) · 박스입수·유통기한 확인 필요</t>
+          <t>※ 직매입 · 냉장 4℃ · 무가당 플레인(과세) · 매가·원가 제안(안) · 유통기한 확인 필요</t>
         </is>
       </c>
     </row>

</xml_diff>